<commit_message>
Client BOM updated with the correct Dupont cable
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Client BOM.xlsx
+++ b/Deliverables/BOM/Client BOM.xlsx
@@ -1,20 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisanderson-tensiondevice\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4581E4B6-8018-451B-8C48-C2D8E959EF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -870,19 +882,19 @@
     <t>JST Cable</t>
   </si>
   <si>
-    <t>7 Pin 15cm Double head inter-connection cable</t>
-  </si>
-  <si>
     <t>Alibaba</t>
   </si>
   <si>
     <t>2.42 inch White OLED</t>
+  </si>
+  <si>
+    <t>7 Pin 10cm Reverse Side Double head inter-connection cable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1383,24 +1395,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K63"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1413,7 +1425,7 @@
       <c r="J1" s="16"/>
       <c r="K1" s="16"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1446,7 +1458,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1478,7 +1490,7 @@
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B58" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1510,7 +1522,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1542,7 +1554,7 @@
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1574,7 +1586,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1606,7 +1618,7 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1638,7 +1650,7 @@
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1670,7 +1682,7 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1702,7 +1714,7 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1734,7 +1746,7 @@
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1766,7 +1778,7 @@
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1798,7 +1810,7 @@
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1830,7 +1842,7 @@
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1862,7 +1874,7 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1894,7 +1906,7 @@
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1926,7 +1938,7 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1958,7 +1970,7 @@
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1990,7 +2002,7 @@
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -2022,7 +2034,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -2054,7 +2066,7 @@
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -2086,7 +2098,7 @@
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -2118,7 +2130,7 @@
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -2150,7 +2162,7 @@
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -2182,7 +2194,7 @@
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -2214,7 +2226,7 @@
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -2246,7 +2258,7 @@
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -2278,7 +2290,7 @@
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -2310,7 +2322,7 @@
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2342,7 +2354,7 @@
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2374,7 +2386,7 @@
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2406,7 +2418,7 @@
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2438,7 +2450,7 @@
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2470,7 +2482,7 @@
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2502,7 +2514,7 @@
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2534,7 +2546,7 @@
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -2566,7 +2578,7 @@
       </c>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -2598,7 +2610,7 @@
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -2630,7 +2642,7 @@
       </c>
       <c r="K39" s="7"/>
     </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f t="shared" si="0"/>
@@ -2662,7 +2674,7 @@
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -2694,7 +2706,7 @@
       </c>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f t="shared" si="0"/>
@@ -2726,7 +2738,7 @@
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
@@ -2758,7 +2770,7 @@
       </c>
       <c r="K43" s="7"/>
     </row>
-    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -2790,7 +2802,7 @@
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
@@ -2822,7 +2834,7 @@
       </c>
       <c r="K45" s="7"/>
     </row>
-    <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
@@ -2854,7 +2866,7 @@
       </c>
       <c r="K46" s="9"/>
     </row>
-    <row r="47" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
@@ -2886,7 +2898,7 @@
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -2918,7 +2930,7 @@
       </c>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
@@ -2950,7 +2962,7 @@
       </c>
       <c r="K49" s="7"/>
     </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
@@ -2982,7 +2994,7 @@
       </c>
       <c r="K50" s="9"/>
     </row>
-    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
@@ -3014,7 +3026,7 @@
       </c>
       <c r="K51" s="7"/>
     </row>
-    <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
         <f t="shared" si="0"/>
@@ -3046,7 +3058,7 @@
       </c>
       <c r="K52" s="9"/>
     </row>
-    <row r="53" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
         <f>ROW(B53) - ROW($B$2)</f>
@@ -3076,7 +3088,7 @@
       </c>
       <c r="K53" s="7"/>
     </row>
-    <row r="54" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
         <f t="shared" si="0"/>
@@ -3108,7 +3120,7 @@
       </c>
       <c r="K54" s="9"/>
     </row>
-    <row r="55" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
         <f>ROW(B55) - ROW($B$2)</f>
@@ -3140,7 +3152,7 @@
       </c>
       <c r="K55" s="7"/>
     </row>
-    <row r="56" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
         <f t="shared" si="0"/>
@@ -3172,7 +3184,7 @@
       </c>
       <c r="K56" s="9"/>
     </row>
-    <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
         <f>ROW(B57) - ROW($B$2)</f>
@@ -3204,7 +3216,7 @@
       </c>
       <c r="K57" s="7"/>
     </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
         <f t="shared" si="0"/>
@@ -3236,7 +3248,7 @@
       </c>
       <c r="K58" s="9"/>
     </row>
-    <row r="59" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
         <f>ROW(B59) - ROW($B$2)</f>
@@ -3268,7 +3280,7 @@
       </c>
       <c r="K59" s="7"/>
     </row>
-    <row r="60" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="11">
         <f>ROW(B60) - ROW($B$2)</f>
         <v>58</v>
@@ -3301,7 +3313,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="11">
         <f t="shared" ref="B61:B63" si="1">ROW(B61) - ROW($B$2)</f>
         <v>59</v>
@@ -3334,7 +3346,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="11">
         <f>ROW(B62) - ROW($B$2)</f>
         <v>60</v>
@@ -3346,7 +3358,7 @@
         <v>273</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>273</v>
@@ -3364,10 +3376,10 @@
         <v>1</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B63" s="11">
         <f t="shared" si="1"/>
         <v>61</v>
@@ -3379,7 +3391,7 @@
         <v>273</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>273</v>
@@ -3405,10 +3417,10 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K60" r:id="rId1"/>
-    <hyperlink ref="K61" r:id="rId2"/>
-    <hyperlink ref="K63" r:id="rId3"/>
-    <hyperlink ref="K62" r:id="rId4"/>
+    <hyperlink ref="K60" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K61" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="K63" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="K62" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>

</xml_diff>